<commit_message>
Dokumentácia: požiadavky bez ovládania a stavov, úrovne AI a bossovia, učenie AI, boj rozpísaný do use cases
</commit_message>
<xml_diff>
--- a/01_Poziadavky/nefunkcionalne-poziadavky.xlsx
+++ b/01_Poziadavky/nefunkcionalne-poziadavky.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Papo\source\repos\Rocnikovy_stick_fight\dokumentacia\Stickops\01_Poziadavky\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9A462ED-BAAC-48FC-8A59-6B4872C025DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A30BA957-3079-4CC0-AC6A-A45249C62D39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3AF123A7-36BC-48C7-99B3-CC8AE1205725}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{082E2884-6E36-47C3-9686-200F8ADF0D0F}"/>
   </bookViews>
   <sheets>
     <sheet name="Nefunkcionálne" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="61">
   <si>
     <t>ID</t>
   </si>
@@ -50,9 +50,6 @@
     <t>MoSCoW</t>
   </si>
   <si>
-    <t>Stav (16. 10. 2026)</t>
-  </si>
-  <si>
     <t>Výkonnosť</t>
   </si>
   <si>
@@ -65,33 +62,24 @@
     <t>M</t>
   </si>
   <si>
-    <t>Hotové – pevný krok simulácie 60 Hz</t>
-  </si>
-  <si>
     <t>NFR-P-02</t>
   </si>
   <si>
-    <t>Systém by mal spracovať stlačenie klávesu najneskôr v nasledujúcej snímke (do 17 ms).</t>
+    <t>Systém by mal spracovať vstup hráča najneskôr v nasledujúcej snímke (do 17 ms).</t>
   </si>
   <si>
     <t>S</t>
   </si>
   <si>
-    <t>Hotové</t>
-  </si>
-  <si>
     <t>NFR-P-03</t>
   </si>
   <si>
-    <t>Systém by mohol pri tréningu AI simulovať zápasy mnohonásobne rýchlejšie ako v reálnom čase (bez grafiky).</t>
+    <t>Systém by mohol pri tréningu AI simulovať zápasy mnohonásobne rýchlejšie ako v reálnom čase.</t>
   </si>
   <si>
     <t>C</t>
   </si>
   <si>
-    <t>Hotové – headless simulácia</t>
-  </si>
-  <si>
     <t>NFR-P-04</t>
   </si>
   <si>
@@ -101,9 +89,6 @@
     <t>W</t>
   </si>
   <si>
-    <t>–</t>
-  </si>
-  <si>
     <t>Dostupnosť</t>
   </si>
   <si>
@@ -122,10 +107,7 @@
     <t>NFR-A-03</t>
   </si>
   <si>
-    <t>Systém by mohol ukladať postup tak, aby ho výpadok nepoškodil.</t>
-  </si>
-  <si>
-    <t>Čiastočne – poškodený postup sa nahradí novým</t>
+    <t>Systém by mohol ukladať postup tak, aby ho výpadok počas ukladania nepoškodil.</t>
   </si>
   <si>
     <t>NFR-A-04</t>
@@ -146,7 +128,7 @@
     <t>NFR-S-02</t>
   </si>
   <si>
-    <t>Systém by mal obsah čítať iba ako dáta – súbory obsahu nespúšťajú kód.</t>
+    <t>Systém by mal súbory obsahu čítať iba ako dáta – nesmú spúšťať kód.</t>
   </si>
   <si>
     <t>NFR-S-03</t>
@@ -182,9 +164,6 @@
     <t>Systém by mohol obsahovať tutoriál pre nového hráča.</t>
   </si>
   <si>
-    <t>Nerealizované – úlohu plní 1. kapitola kampane (Tréningová hala)</t>
-  </si>
-  <si>
     <t>NFR-U-04</t>
   </si>
   <si>
@@ -197,13 +176,13 @@
     <t>NFR-SC-01</t>
   </si>
   <si>
-    <t>Systém musí umožniť pridať arénu, útok, finisher alebo osobnosť AI iba pridaním súboru JSON.</t>
+    <t>Systém musí umožniť pridať arénu, útok, finisher alebo súpera AI iba pridaním súboru JSON.</t>
   </si>
   <si>
     <t>NFR-SC-02</t>
   </si>
   <si>
-    <t>Systém by mal zvládnuť rozšírenie kampane nad 25 levelov bez zmeny kódu (campaign.json).</t>
+    <t>Systém by mal zvládnuť rozšírenie kampane nad 25 levelov bez zmeny kódu.</t>
   </si>
   <si>
     <t>NFR-SC-03</t>
@@ -212,9 +191,6 @@
     <t>Systém by mohol umožniť boj viac ako dvoch bojovníkov naraz.</t>
   </si>
   <si>
-    <t>Nerealizované – presily sú súperi po sebe</t>
-  </si>
-  <si>
     <t>NFR-SC-04</t>
   </si>
   <si>
@@ -227,28 +203,19 @@
     <t>NFR-B-01</t>
   </si>
   <si>
-    <t>Systém musí mať herné pravidlá oddelené od kreslenia a deterministickú simuláciu.</t>
-  </si>
-  <si>
-    <t>Hotové – game/src/core, overené testami determinizmu a replayov</t>
+    <t>Systém musí mať herné pravidlá oddelené od kreslenia a deterministickú simuláciu (rovnaké vstupy = rovnaký výsledok).</t>
   </si>
   <si>
     <t>NFR-B-02</t>
   </si>
   <si>
-    <t>Systém by mal mať automatické testy (doctest).</t>
-  </si>
-  <si>
-    <t>Hotové – stick_tests.exe a stick_ai_tests.exe</t>
+    <t>Systém by mal mať automatické testy.</t>
   </si>
   <si>
     <t>NFR-B-03</t>
   </si>
   <si>
-    <t>Systém by mohol mať dokumentáciu formátu obsahu.</t>
-  </si>
-  <si>
-    <t>Hotové – game/content/README.md, docs/pre-dizajnera.md</t>
+    <t>Systém by mohol mať dokumentáciu formátu súborov obsahu.</t>
   </si>
   <si>
     <t>NFR-B-04</t>
@@ -678,17 +645,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E7823B-CA8B-4F8E-B251-58B2266B7767}">
-  <dimension ref="A1:D31"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10C94E8E-5CA2-4E1C-813B-187FD704157E}">
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
-    <col min="2" max="2" width="80.7109375" customWidth="1"/>
+    <col min="2" max="2" width="95.7109375" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" customWidth="1"/>
-    <col min="4" max="4" width="45.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -698,392 +664,311 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="3" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C10" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="C15" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="C20" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-    </row>
-    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-    </row>
-    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C30" s="3" t="s">
+      <c r="C31" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>